<commit_message>
feat: add types for map features including counties, parishes, resources, and hydrography
</commit_message>
<xml_diff>
--- a/fixtures/sample-ari.xlsx
+++ b/fixtures/sample-ari.xlsx
@@ -8,6 +8,20 @@
     <sheet name="Subnets" sheetId="3" r:id="rId3"/>
     <sheet name="Network Interface" sheetId="4" r:id="rId4"/>
     <sheet name="VNET Peerings" sheetId="5" r:id="rId5"/>
+    <sheet name="Storage Accounts" sheetId="6" r:id="rId6"/>
+    <sheet name="Key Vaults" sheetId="7" r:id="rId7"/>
+    <sheet name="SQL Databases" sheetId="8" r:id="rId8"/>
+    <sheet name="App Services" sheetId="9" r:id="rId9"/>
+    <sheet name="Function Apps" sheetId="10" r:id="rId10"/>
+    <sheet name="AKS" sheetId="11" r:id="rId11"/>
+    <sheet name="Application Gateways" sheetId="12" r:id="rId12"/>
+    <sheet name="Event Hubs" sheetId="13" r:id="rId13"/>
+    <sheet name="Service Bus" sheetId="14" r:id="rId14"/>
+    <sheet name="Log Analytics" sheetId="15" r:id="rId15"/>
+    <sheet name="Public IP Addresses" sheetId="16" r:id="rId16"/>
+    <sheet name="ExpressRoute Circuits" sheetId="17" r:id="rId17"/>
+    <sheet name="Virtual Network Gateways" sheetId="18" r:id="rId18"/>
+    <sheet name="Role Assignments" sheetId="19" r:id="rId19"/>
   </sheets>
 </workbook>
 </file>
@@ -401,7 +415,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:G10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -422,6 +436,9 @@
       <c r="F1" t="str">
         <v>Subscription</v>
       </c>
+      <c r="G1" t="str">
+        <v>Tags</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -440,7 +457,10 @@
         <v>Linux</v>
       </c>
       <c r="F2" t="str">
-        <v>demo-sub</v>
+        <v>Production</v>
+      </c>
+      <c r="G2" t="str">
+        <v>environment=production;tier=web</v>
       </c>
     </row>
     <row r="3">
@@ -460,7 +480,10 @@
         <v>Linux</v>
       </c>
       <c r="F3" t="str">
-        <v>demo-sub</v>
+        <v>Production</v>
+      </c>
+      <c r="G3" t="str">
+        <v>environment=production;tier=web</v>
       </c>
     </row>
     <row r="4">
@@ -480,7 +503,10 @@
         <v>Linux</v>
       </c>
       <c r="F4" t="str">
-        <v>demo-sub</v>
+        <v>Production</v>
+      </c>
+      <c r="G4" t="str">
+        <v>environment=production;tier=app</v>
       </c>
     </row>
     <row r="5">
@@ -500,7 +526,10 @@
         <v>Linux</v>
       </c>
       <c r="F5" t="str">
-        <v>demo-sub</v>
+        <v>Production</v>
+      </c>
+      <c r="G5" t="str">
+        <v>environment=production;tier=app</v>
       </c>
     </row>
     <row r="6">
@@ -520,7 +549,10 @@
         <v>Linux</v>
       </c>
       <c r="F6" t="str">
-        <v>demo-sub</v>
+        <v>Production</v>
+      </c>
+      <c r="G6" t="str">
+        <v>environment=production;tier=data</v>
       </c>
     </row>
     <row r="7">
@@ -540,7 +572,10 @@
         <v>Linux</v>
       </c>
       <c r="F7" t="str">
-        <v>demo-sub</v>
+        <v>Production</v>
+      </c>
+      <c r="G7" t="str">
+        <v>environment=production;tier=data</v>
       </c>
     </row>
     <row r="8">
@@ -548,7 +583,7 @@
         <v>win-01</v>
       </c>
       <c r="B8" t="str">
-        <v>rg-corp</v>
+        <v>rg-dev</v>
       </c>
       <c r="C8" t="str">
         <v>northeurope</v>
@@ -560,7 +595,10 @@
         <v>Windows</v>
       </c>
       <c r="F8" t="str">
-        <v>demo-sub</v>
+        <v>Development</v>
+      </c>
+      <c r="G8" t="str">
+        <v>environment=development</v>
       </c>
     </row>
     <row r="9">
@@ -568,7 +606,7 @@
         <v>win-02</v>
       </c>
       <c r="B9" t="str">
-        <v>rg-corp</v>
+        <v>rg-dev</v>
       </c>
       <c r="C9" t="str">
         <v>northeurope</v>
@@ -580,7 +618,10 @@
         <v>Windows</v>
       </c>
       <c r="F9" t="str">
-        <v>demo-sub</v>
+        <v>Development</v>
+      </c>
+      <c r="G9" t="str">
+        <v>environment=development</v>
       </c>
     </row>
     <row r="10">
@@ -588,7 +629,7 @@
         <v>jump</v>
       </c>
       <c r="B10" t="str">
-        <v>rg-corp</v>
+        <v>rg-dev</v>
       </c>
       <c r="C10" t="str">
         <v>northeurope</v>
@@ -600,19 +641,873 @@
         <v>Windows</v>
       </c>
       <c r="F10" t="str">
-        <v>demo-sub</v>
+        <v>Development</v>
+      </c>
+      <c r="G10" t="str">
+        <v>environment=development</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G10"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Resource Group</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Location</v>
+      </c>
+      <c r="D1" t="str">
+        <v>SKU</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Subscription</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Tags</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>func-events</v>
+      </c>
+      <c r="B2" t="str">
+        <v>rg-app</v>
+      </c>
+      <c r="C2" t="str">
+        <v>westeurope</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Y1</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Production</v>
+      </c>
+      <c r="F2" t="str">
+        <v>environment=production;tier=app</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>func-dev</v>
+      </c>
+      <c r="B3" t="str">
+        <v>rg-dev</v>
+      </c>
+      <c r="C3" t="str">
+        <v>northeurope</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Y1</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Development</v>
+      </c>
+      <c r="F3" t="str">
+        <v>environment=development</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Resource Group</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Location</v>
+      </c>
+      <c r="D1" t="str">
+        <v>VM Size</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Node Count</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Kubernetes Version</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Subscription</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Tags</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>aks-prod</v>
+      </c>
+      <c r="B2" t="str">
+        <v>rg-app</v>
+      </c>
+      <c r="C2" t="str">
+        <v>westeurope</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Standard_D4s_v3</v>
+      </c>
+      <c r="E2">
+        <v>4</v>
+      </c>
+      <c r="F2" t="str">
+        <v>1.29</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Production</v>
+      </c>
+      <c r="H2" t="str">
+        <v>environment=production;tier=app</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Resource Group</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Location</v>
+      </c>
+      <c r="D1" t="str">
+        <v>SKU</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Tier</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Subscription</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Tags</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>agw-prod</v>
+      </c>
+      <c r="B2" t="str">
+        <v>rg-infra</v>
+      </c>
+      <c r="C2" t="str">
+        <v>westeurope</v>
+      </c>
+      <c r="D2" t="str">
+        <v>WAF_v2</v>
+      </c>
+      <c r="E2" t="str">
+        <v>WAF_v2</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Shared Services</v>
+      </c>
+      <c r="G2" t="str">
+        <v>environment=production</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Resource Group</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Location</v>
+      </c>
+      <c r="D1" t="str">
+        <v>SKU</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Subscription</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Tags</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>evh-prod-ingest</v>
+      </c>
+      <c r="B2" t="str">
+        <v>rg-app</v>
+      </c>
+      <c r="C2" t="str">
+        <v>westeurope</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Standard</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Production</v>
+      </c>
+      <c r="F2" t="str">
+        <v>environment=production;tier=app</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>evh-prod-telemetry</v>
+      </c>
+      <c r="B3" t="str">
+        <v>rg-data</v>
+      </c>
+      <c r="C3" t="str">
+        <v>westeurope</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Standard</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Production</v>
+      </c>
+      <c r="F3" t="str">
+        <v>environment=production;tier=data</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>evh-dev</v>
+      </c>
+      <c r="B4" t="str">
+        <v>rg-dev</v>
+      </c>
+      <c r="C4" t="str">
+        <v>northeurope</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Basic</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Development</v>
+      </c>
+      <c r="F4" t="str">
+        <v>environment=development</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Resource Group</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Location</v>
+      </c>
+      <c r="D1" t="str">
+        <v>SKU</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Subscription</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Tags</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>sb-prod-orders</v>
+      </c>
+      <c r="B2" t="str">
+        <v>rg-app</v>
+      </c>
+      <c r="C2" t="str">
+        <v>westeurope</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Standard</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Production</v>
+      </c>
+      <c r="F2" t="str">
+        <v>environment=production;tier=app</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>sb-prod-notify</v>
+      </c>
+      <c r="B3" t="str">
+        <v>rg-app</v>
+      </c>
+      <c r="C3" t="str">
+        <v>westeurope</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Premium</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Production</v>
+      </c>
+      <c r="F3" t="str">
+        <v>environment=production;tier=app</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Resource Group</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Location</v>
+      </c>
+      <c r="D1" t="str">
+        <v>SKU</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Subscription</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Tags</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>log-shared-central</v>
+      </c>
+      <c r="B2" t="str">
+        <v>rg-infra</v>
+      </c>
+      <c r="C2" t="str">
+        <v>westeurope</v>
+      </c>
+      <c r="D2" t="str">
+        <v>PerGB2018</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Shared Services</v>
+      </c>
+      <c r="F2" t="str">
+        <v>environment=production</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>log-dev</v>
+      </c>
+      <c r="B3" t="str">
+        <v>rg-dev</v>
+      </c>
+      <c r="C3" t="str">
+        <v>northeurope</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Free</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Development</v>
+      </c>
+      <c r="F3" t="str">
+        <v>environment=development</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Resource Group</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Location</v>
+      </c>
+      <c r="D1" t="str">
+        <v>SKU</v>
+      </c>
+      <c r="E1" t="str">
+        <v>IP Address</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Subscription</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Tags</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>pip-agw-prod</v>
+      </c>
+      <c r="B2" t="str">
+        <v>rg-infra</v>
+      </c>
+      <c r="C2" t="str">
+        <v>westeurope</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Standard</v>
+      </c>
+      <c r="E2" t="str">
+        <v>51.105.22.10</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Shared Services</v>
+      </c>
+      <c r="G2" t="str">
+        <v>environment=production</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>pip-vpngw-prod</v>
+      </c>
+      <c r="B3" t="str">
+        <v>rg-network</v>
+      </c>
+      <c r="C3" t="str">
+        <v>westeurope</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Standard</v>
+      </c>
+      <c r="E3" t="str">
+        <v>51.105.22.11</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Production</v>
+      </c>
+      <c r="G3" t="str">
+        <v>environment=production</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>pip-bastion</v>
+      </c>
+      <c r="B4" t="str">
+        <v>rg-infra</v>
+      </c>
+      <c r="C4" t="str">
+        <v>westeurope</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Standard</v>
+      </c>
+      <c r="E4" t="str">
+        <v>51.105.22.12</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Shared Services</v>
+      </c>
+      <c r="G4" t="str">
+        <v>environment=production</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Resource Group</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Location</v>
+      </c>
+      <c r="D1" t="str">
+        <v>SKU</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Bandwidth (Mbps)</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Provider</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Subscription</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Tags</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>er-corp-london</v>
+      </c>
+      <c r="B2" t="str">
+        <v>rg-network</v>
+      </c>
+      <c r="C2" t="str">
+        <v>westeurope</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Standard</v>
+      </c>
+      <c r="E2" t="str">
+        <v>1000</v>
+      </c>
+      <c r="F2" t="str">
+        <v>BT</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Production</v>
+      </c>
+      <c r="H2" t="str">
+        <v>environment=production</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Resource Group</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Location</v>
+      </c>
+      <c r="D1" t="str">
+        <v>SKU</v>
+      </c>
+      <c r="E1" t="str">
+        <v>VPN Type</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Subscription</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Tags</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>vpngw-prod</v>
+      </c>
+      <c r="B2" t="str">
+        <v>rg-network</v>
+      </c>
+      <c r="C2" t="str">
+        <v>westeurope</v>
+      </c>
+      <c r="D2" t="str">
+        <v>VpnGw2</v>
+      </c>
+      <c r="E2" t="str">
+        <v>RouteBased</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Production</v>
+      </c>
+      <c r="G2" t="str">
+        <v>environment=production</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>vpngw-dev</v>
+      </c>
+      <c r="B3" t="str">
+        <v>rg-network</v>
+      </c>
+      <c r="C3" t="str">
+        <v>northeurope</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Basic</v>
+      </c>
+      <c r="E3" t="str">
+        <v>RouteBased</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Development</v>
+      </c>
+      <c r="G3" t="str">
+        <v>environment=development</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Principal Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Principal Type</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Role Definition Name</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Subscription</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Resource Group</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>ops-team</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Group</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Contributor</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Production</v>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>devops-sp</v>
+      </c>
+      <c r="B3" t="str">
+        <v>ServicePrincipal</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Owner</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Production</v>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>audit-reader</v>
+      </c>
+      <c r="B4" t="str">
+        <v>User</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Reader</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Shared Services</v>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>dev-team</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Group</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Contributor</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Development</v>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>sec-auditor</v>
+      </c>
+      <c r="B6" t="str">
+        <v>User</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Reader</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Production</v>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>data-engineers</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Group</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Owner</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Production</v>
+      </c>
+      <c r="E7" t="str">
+        <v>rg-data</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>frontend-devs</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Group</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Contributor</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Production</v>
+      </c>
+      <c r="E8" t="str">
+        <v>rg-frontend</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>readonly-bot</v>
+      </c>
+      <c r="B9" t="str">
+        <v>ServicePrincipal</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Reader</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Production</v>
+      </c>
+      <c r="E9" t="str">
+        <v>rg-app</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>junior-devs</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Group</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Reader</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Development</v>
+      </c>
+      <c r="E10" t="str">
+        <v>rg-dev</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:E4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -627,6 +1522,9 @@
       <c r="D1" t="str">
         <v>Address Space</v>
       </c>
+      <c r="E1" t="str">
+        <v>Subscription</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -641,31 +1539,54 @@
       <c r="D2" t="str">
         <v>10.0.0.0/16</v>
       </c>
+      <c r="E2" t="str">
+        <v>Production</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>vnet-corp</v>
+        <v>vnet-shared</v>
       </c>
       <c r="B3" t="str">
         <v>rg-network</v>
       </c>
       <c r="C3" t="str">
+        <v>westeurope</v>
+      </c>
+      <c r="D3" t="str">
+        <v>10.2.0.0/16</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Shared Services</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>vnet-corp</v>
+      </c>
+      <c r="B4" t="str">
+        <v>rg-network</v>
+      </c>
+      <c r="C4" t="str">
         <v>northeurope</v>
       </c>
-      <c r="D3" t="str">
+      <c r="D4" t="str">
         <v>10.1.0.0/16</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Development</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -713,18 +1634,29 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
+        <v>vnet-shared</v>
+      </c>
+      <c r="B5" t="str">
+        <v>snet-infra</v>
+      </c>
+      <c r="C5" t="str">
+        <v>10.2.1.0/24</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
         <v>vnet-corp</v>
       </c>
-      <c r="B5" t="str">
+      <c r="B6" t="str">
         <v>snet-corp</v>
       </c>
-      <c r="C5" t="str">
+      <c r="C6" t="str">
         <v>10.1.1.0/24</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -912,7 +1844,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -930,15 +1862,360 @@
         <v>vnet-prod</v>
       </c>
       <c r="B2" t="str">
-        <v>vnet-corp</v>
+        <v>vnet-shared</v>
       </c>
       <c r="C2" t="str">
         <v>Connected</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>vnet-prod</v>
+      </c>
+      <c r="B3" t="str">
+        <v>vnet-corp</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Connected</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Resource Group</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Location</v>
+      </c>
+      <c r="D1" t="str">
+        <v>SKU</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Kind</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Subscription</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Tags</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>stfrontend</v>
+      </c>
+      <c r="B2" t="str">
+        <v>rg-frontend</v>
+      </c>
+      <c r="C2" t="str">
+        <v>westeurope</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Standard_LRS</v>
+      </c>
+      <c r="E2" t="str">
+        <v>StorageV2</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Production</v>
+      </c>
+      <c r="G2" t="str">
+        <v>environment=production</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>stdatalake</v>
+      </c>
+      <c r="B3" t="str">
+        <v>rg-data</v>
+      </c>
+      <c r="C3" t="str">
+        <v>westeurope</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Standard_GRS</v>
+      </c>
+      <c r="E3" t="str">
+        <v>StorageV2</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Production</v>
+      </c>
+      <c r="G3" t="str">
+        <v>environment=production;tier=data</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>stdev</v>
+      </c>
+      <c r="B4" t="str">
+        <v>rg-dev</v>
+      </c>
+      <c r="C4" t="str">
+        <v>northeurope</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Standard_LRS</v>
+      </c>
+      <c r="E4" t="str">
+        <v>BlobStorage</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Development</v>
+      </c>
+      <c r="G4" t="str">
+        <v>environment=development</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Resource Group</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Location</v>
+      </c>
+      <c r="D1" t="str">
+        <v>SKU</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Subscription</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Tags</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>kv-prod-main</v>
+      </c>
+      <c r="B2" t="str">
+        <v>rg-infra</v>
+      </c>
+      <c r="C2" t="str">
+        <v>westeurope</v>
+      </c>
+      <c r="D2" t="str">
+        <v>premium</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Shared Services</v>
+      </c>
+      <c r="F2" t="str">
+        <v>environment=production</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>kv-prod-data</v>
+      </c>
+      <c r="B3" t="str">
+        <v>rg-data</v>
+      </c>
+      <c r="C3" t="str">
+        <v>westeurope</v>
+      </c>
+      <c r="D3" t="str">
+        <v>standard</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Production</v>
+      </c>
+      <c r="F3" t="str">
+        <v>environment=production;tier=data</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Resource Group</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Location</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Server</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Tier</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Subscription</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Tags</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>sql-app-db</v>
+      </c>
+      <c r="B2" t="str">
+        <v>rg-app</v>
+      </c>
+      <c r="C2" t="str">
+        <v>westeurope</v>
+      </c>
+      <c r="D2" t="str">
+        <v>sql-prod-server</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Standard S2</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Production</v>
+      </c>
+      <c r="G2" t="str">
+        <v>environment=production;tier=app</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>sql-dw</v>
+      </c>
+      <c r="B3" t="str">
+        <v>rg-data</v>
+      </c>
+      <c r="C3" t="str">
+        <v>westeurope</v>
+      </c>
+      <c r="D3" t="str">
+        <v>sql-prod-server</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Premium P1</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Production</v>
+      </c>
+      <c r="G3" t="str">
+        <v>environment=production;tier=data</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Resource Group</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Location</v>
+      </c>
+      <c r="D1" t="str">
+        <v>SKU</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Kind</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Subscription</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Tags</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>app-frontend</v>
+      </c>
+      <c r="B2" t="str">
+        <v>rg-frontend</v>
+      </c>
+      <c r="C2" t="str">
+        <v>westeurope</v>
+      </c>
+      <c r="D2" t="str">
+        <v>B2</v>
+      </c>
+      <c r="E2" t="str">
+        <v>app</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Production</v>
+      </c>
+      <c r="G2" t="str">
+        <v>environment=production</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>app-api</v>
+      </c>
+      <c r="B3" t="str">
+        <v>rg-app</v>
+      </c>
+      <c r="C3" t="str">
+        <v>westeurope</v>
+      </c>
+      <c r="D3" t="str">
+        <v>P2v3</v>
+      </c>
+      <c r="E3" t="str">
+        <v>app</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Production</v>
+      </c>
+      <c r="G3" t="str">
+        <v>environment=production;tier=app</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>